<commit_message>
docs(sen0308): add provisional 3523g reading and reject unstable block
</commit_message>
<xml_diff>
--- a/docs/Calibration_SEN0308.xlsx
+++ b/docs/Calibration_SEN0308.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Données CR1000" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Points calibration'!$A$4:$J$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Points calibration'!$A$4:$J$17</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -500,7 +500,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -586,12 +586,12 @@
     <row r="9" ht="42" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Pesée ultérieure</t>
+          <t>Pesée précédente</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Pot pesé à 3 530 g le 15/10 : 1 480 g au-dessus de la référence sèche, soit 30,83 % vol. Aucun relevé mV exactement associé à cette pesée n’est confirmé.</t>
+          <t>Pot pesé à 3 530 g le 15/10 : 1 480 g au-dessus de la référence sèche, soit 30,83 % vol. Pas de moyenne mV exactement associée à cette pesée.</t>
         </is>
       </c>
     </row>
@@ -631,97 +631,123 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="30" customHeight="1">
+    <row r="13" ht="42" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Dernière fenêtre exportée</t>
+          <t>Mesure actuelle — provisoire</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>15/10 14:40–14:45 : 1819.65 mV. Non validée : dernier bloc instable (écart-type 15.66 mV) et poids correspondant non enregistré.</t>
+          <t>Poids déclaré : 3523 g. Fenêtre stable 15/10 14:39:30–14:44:30 : 1822.88 mV (10 blocs, écart-type estimé 0.75 mV). θ apparente = 30.69 % vol.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="42" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
         <is>
+          <t>Contrôle de cohérence</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>La masse actuelle est seulement 32 g sous la capacité au champ, mais le signal diffère de 302.7 mV. Point à vérifier (même profondeur/contact, pot et câble pesés de la même façon) ; ne pas encore l’utiliser dans l’ajustement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Bloc final rejeté</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Le dernier enregistrement du fichier est 2026-10-15 14:45:00 : 1790.56 mV, écart-type 15.66 mV. Il est exclu de la moyenne stable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="42" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
           <t>État de calibration</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Deux points interprétables sont consignés (terreau sec et capacité au champ). Ils ne suffisent pas à valider une loi θ = f(mV) ; ajouter des points intermédiaires pendant le dessèchement.</t>
+          <t>Deux références restent utilisables (terreau sec et capacité au champ). Le nouveau couple poids/mV est conservé comme provisoire, car sa variation de signal paraît incohérente avec l’écart de masse.</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="42" customHeight="1">
-      <c r="A15" s="3" t="inlineStr">
+    <row r="17" ht="42" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>Prochain point utile</t>
         </is>
       </c>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>Laisser sécher sans ajouter d’eau. Pour une baisse d’environ 10 % vol. depuis la capacité au champ : viser ≈ 3 075 g pot+terreau (sans sonde), puis noter la masse et la moyenne mV sur une fenêtre stable de 5 min.</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="42" customHeight="1">
-      <c r="A16" s="3" t="inlineStr">
+    <row r="18" ht="42" customHeight="1">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>Comment ajouter un relevé</t>
         </is>
       </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>Dans « Points calibration », saisir une ligne avec le poids du pot sans sonde, la date/heure, la moyenne SEN_mV sur 5 min et le plus grand écart-type des blocs. Les colonnes d’eau retenue et θ sont calculées automatiquement.</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="42" customHeight="1">
-      <c r="A17" s="3" t="inlineStr">
+    <row r="19" ht="42" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>Attention au champ Point</t>
         </is>
       </c>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Le programme a gardé Point=6 du 14/10 au 15/10. Ce numéro ne prouve pas que toutes ces lignes sont au même état d’humidité : utiliser poids + heure pour identifier les étapes. La dernière fenêtre est signalée, pas utilisée comme point de calibration.</t>
+          <t>Le programme a gardé Point=6 du 14/10 au 15/10. Ce numéro ne prouve pas que toutes ces lignes sont au même état d’humidité : utiliser poids + heure pour identifier les étapes. Le bloc de 14:45 est exclu.</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="3" t="inlineStr">
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="3" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <t>D:\Mes Programmes\CR1000calibsonde_CalibSEN0308.dat</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="17">
+  <mergeCells count="19">
+    <mergeCell ref="B11:D11"/>
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="B13:D13"/>
     <mergeCell ref="B10:D10"/>
+    <mergeCell ref="B19:D19"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="B15:D15"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="B20:D20"/>
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="B11:D11"/>
     <mergeCell ref="B5:D5"/>
-    <mergeCell ref="B14:D14"/>
-    <mergeCell ref="B15:D15"/>
-    <mergeCell ref="B8:D8"/>
     <mergeCell ref="B4:D4"/>
-    <mergeCell ref="B17:D17"/>
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="B16:D16"/>
     <mergeCell ref="B18:D18"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="B12:D12"/>
-    <mergeCell ref="B7:D7"/>
-    <mergeCell ref="B6:D6"/>
-    <mergeCell ref="B16:D16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -733,7 +759,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:J17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -931,15 +957,17 @@
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
         <is>
-          <t>Observation export, non validée</t>
+          <t>6 — séchage, à vérifier</t>
         </is>
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>15/10/2026 14:40–14:45</t>
+          <t>15/10/2026 14:39:30–14:44:30</t>
         </is>
       </c>
-      <c r="C8" s="10" t="n"/>
+      <c r="C8" s="10" t="n">
+        <v>3523</v>
+      </c>
       <c r="D8" s="10" t="n">
         <v>2050</v>
       </c>
@@ -952,58 +980,62 @@
         <v/>
       </c>
       <c r="G8" s="12" t="n">
-        <v>1819.6523</v>
+        <v>1822.8837</v>
       </c>
       <c r="H8" s="12" t="n">
-        <v>10.9129707066448</v>
+        <v>0.7540599357683513</v>
       </c>
       <c r="I8" s="9" t="n">
         <v>10</v>
       </c>
       <c r="J8" s="9" t="inlineStr">
         <is>
-          <t>À exclure de l’ajustement : bloc final instable (Std max 15.66 mV), poids inconnu.</t>
+          <t>Couple déclaré 3 523 g / 1822.88 mV ; provisoire : +302.7 mV pour seulement -32 g vs capacité au champ.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="9" t="inlineStr">
+      <c r="A9" t="inlineStr">
         <is>
-          <t>5 — prochain palier visé</t>
+          <t>Bloc isolé, rejeté</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
-          <t>À compléter</t>
+          <t>2026-10-15 14:45:00</t>
         </is>
       </c>
-      <c r="C9" s="10" t="n">
-        <v>3075</v>
-      </c>
-      <c r="D9" s="10" t="n">
+      <c r="C9" s="6" t="n"/>
+      <c r="D9" s="6" t="n">
         <v>2050</v>
       </c>
-      <c r="E9" s="10">
+      <c r="E9" s="6">
         <f>IF(C9="","",C9-D9)</f>
         <v/>
       </c>
-      <c r="F9" s="11">
+      <c r="F9" s="7">
         <f>IF(E9="","",100*E9/4800.0)</f>
         <v/>
       </c>
-      <c r="G9" s="12" t="n"/>
-      <c r="H9" s="12" t="n"/>
-      <c r="I9" s="9" t="n"/>
-      <c r="J9" s="9" t="inlineStr">
+      <c r="G9" s="8" t="n">
+        <v>1790.559</v>
+      </c>
+      <c r="H9" s="8" t="n">
+        <v>15.6609</v>
+      </c>
+      <c r="I9" t="n">
+        <v>1</v>
+      </c>
+      <c r="J9" t="inlineStr">
         <is>
-          <t>Cible indicative, environ 10 % vol. sous capacité au champ ; saisir la vraie pesée et la fenêtre stable.</t>
+          <t>Écart-type élevé au dernier enregistrement ; ne pas utiliser.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
         <is>
-          <t>4 — palier suivant indicatif</t>
+          <t>5 — prochain palier visé</t>
         </is>
       </c>
       <c r="B10" s="9" t="inlineStr">
@@ -1012,7 +1044,7 @@
         </is>
       </c>
       <c r="C10" s="10" t="n">
-        <v>2595</v>
+        <v>3075</v>
       </c>
       <c r="D10" s="10" t="n">
         <v>2050</v>
@@ -1030,18 +1062,24 @@
       <c r="I10" s="9" t="n"/>
       <c r="J10" s="9" t="inlineStr">
         <is>
-          <t>Cible indicative ; saisir la vraie pesée et la fenêtre stable.</t>
+          <t>Cible indicative, environ 10 % vol. sous capacité au champ ; saisir la vraie pesée et la fenêtre stable.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
         <is>
+          <t>4 — palier suivant indicatif</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
           <t>À compléter</t>
         </is>
       </c>
-      <c r="B11" s="9" t="n"/>
-      <c r="C11" s="10" t="n"/>
+      <c r="C11" s="10" t="n">
+        <v>2595</v>
+      </c>
       <c r="D11" s="10" t="n">
         <v>2050</v>
       </c>
@@ -1056,7 +1094,11 @@
       <c r="G11" s="12" t="n"/>
       <c r="H11" s="12" t="n"/>
       <c r="I11" s="9" t="n"/>
-      <c r="J11" s="9" t="n"/>
+      <c r="J11" s="9" t="inlineStr">
+        <is>
+          <t>Cible indicative ; saisir la vraie pesée et la fenêtre stable.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
@@ -1178,8 +1220,32 @@
       <c r="I16" s="9" t="n"/>
       <c r="J16" s="9" t="n"/>
     </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>À compléter</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="n"/>
+      <c r="C17" s="10" t="n"/>
+      <c r="D17" s="10" t="n">
+        <v>2050</v>
+      </c>
+      <c r="E17" s="10">
+        <f>IF(C17="","",C17-D17)</f>
+        <v/>
+      </c>
+      <c r="F17" s="11">
+        <f>IF(E17="","",100*E17/4800.0)</f>
+        <v/>
+      </c>
+      <c r="G17" s="12" t="n"/>
+      <c r="H17" s="12" t="n"/>
+      <c r="I17" s="9" t="n"/>
+      <c r="J17" s="9" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:J16"/>
+  <autoFilter ref="A4:J17"/>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A2:J2"/>

</xml_diff>